<commit_message>
Implement Tier 2 Hybrid Context Generator with CFG
Replaced stub with full in-process Hybrid Context Generator for Repo_Into_Graph_Application. Parses Java/C# code, extracts methods/statements, builds CFG skeleton, identifies critical snippets, and enriches metadata (async, dependencies, exceptions, etc.). Added internal modules: SourceScanner, CodeStructureParser, CfgBuilder, CriticalSnippetExtractor, EnrichedMetadataExtractor, HybridPromptComposer, MermaidRenderer, NodeLabelHumanizer. Updated HybridContextOutputDto with detailed output contract. Refactored DI registration. Enhanced Python benchmark tool for semantic CFG comparison and improved Excel export. Updated .gitignore and test checklist. Enables robust, semantically rich context for LLM code reasoning.
</commit_message>
<xml_diff>
--- a/benchmark_tools/Tang_2_Hybrid_Context/Checklist_Test_Tang_2_Handover.xlsx
+++ b/benchmark_tools/Tang_2_Hybrid_Context/Checklist_Test_Tang_2_Handover.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -641,6 +641,525 @@
       </c>
       <c r="H6" s="4" t="inlineStr"/>
     </row>
+    <row r="7" ht="133.5" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>TC_H_03</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>CFG cho chuoi if / else-if / else va cac diem return som</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>public String classify(int score) {
+    if (score &gt;= 90) {
+        return "A";
+    } else if (score &gt;= 70) {
+        return "B";
+    } else {
+        return "C";
+    }
+}</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>SLOC=9, V(G)=3 -&gt; ROUTE_HYBRID</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>graph TD
+  A[Start] --&gt; B{score &gt;= 90?}
+  B -- Yes --&gt; C[Return A]
+  B -- No --&gt; D{score &gt;= 70?}
+  D -- Yes --&gt; E[Return B]
+  D -- No --&gt; F[Return C]</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>if (score &gt;= 90) {
+if (score &gt;= 70) {</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="187.5" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>TC_H_04</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Vong lap for co continue va break - kiem tra canh quay lui va canh thoat vong lap</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>public int sumPositive(List&lt;Integer&gt; nums) {
+    int total = 0;
+    for (int i = 0; i &lt; nums.size(); i++) {
+        if (nums.get(i) &lt; 0) {
+            continue;
+        }
+        if (total &gt; LIMIT) {
+            break;
+        }
+        total += nums.get(i);
+    }
+    return total;
+}</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>SLOC=12, V(G)=4 -&gt; ROUTE_HYBRID</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>graph TD
+  A[Start] --&gt; B[Set total = 0]
+  B --&gt; C[Init int i = 0]
+  C --&gt; D{Loop while i &lt; nums.size?}
+  D -- Yes --&gt; E{nums.get i &lt; 0?}
+  E -- Yes --&gt; F[Next i++]
+  E -- No --&gt; G{total &gt; LIMIT?}
+  G -- No --&gt; H[Update total]
+  H --&gt; F
+  F --&gt; D
+  D -- No --&gt; I[Return total]</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>for (int i = 0; i &lt; nums.size(); i++) {
+if (nums.get(i) &lt; 0) {
+if (total &gt; LIMIT) {</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="160.5" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>TC_H_05</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Khoi try / catch / finally - canh exception va lenh throw ben trong catch</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>public void charge(Order order) {
+    try {
+        gateway.authorize(order.getId());
+        repository.save(order);
+    } catch (TimeoutException e) {
+        logger.error("timeout", e);
+        throw new PaymentException(e);
+    } finally {
+        lockManager.release(order.getId());
+    }
+}</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>SLOC=10, V(G)=2 -&gt; ROUTE_HYBRID</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>graph TD
+  A[Start] --&gt; B[Try]
+  B --&gt; C[Authorize gateway]
+  C --&gt; D[Save order]
+  B -- exception --&gt; E[Catch Timeout]
+  E --&gt; F[Error logger]
+  F --&gt; G[Throw Payment]
+  D --&gt; H[Finally]
+  H --&gt; I[Release lockManager]</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>catch (TimeoutException e)
+throw new PaymentException(e);</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="147" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>TC_H_06</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Switch nhieu nhanh co default - moi case phai la mot canh rieng</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>public double fee(String type) {
+    switch (type) {
+        case "VIP":
+            return 0;
+        case "NORMAL":
+            return 10;
+        default:
+            return 20;
+    }
+}</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>SLOC=9, V(G)=3 -&gt; ROUTE_HYBRID</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>graph TD
+  A[Start] --&gt; B{Switch on type?}
+  B -- case VIP --&gt; C[Return 0]
+  B -- case NORMAL --&gt; D[Return 10]
+  B -- default --&gt; E[Return 20]</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>switch (type) {</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="174" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>TC_H_07</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Ma nguon C# async/await - nhan dien async marker va khoi using</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>csharp</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>public async Task&lt;Result&gt; SaveAsync(Request request, CancellationToken ct)
+{
+    if (request is null)
+    {
+        throw new ArgumentNullException(nameof(request));
+    }
+    using (var scope = _factory.CreateScope())
+    {
+        var saved = await _repository.SaveAsync(request, ct);
+        return Result.Ok(saved);
+    }
+}</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>SLOC=11, V(G)=2 -&gt; ROUTE_HYBRID</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>graph TD
+  A[Start] --&gt; B{request is null?}
+  B -- Yes --&gt; C[Throw ArgumentNull]
+  B -- No --&gt; D[using var scope = _factory.CreateScope]
+  D --&gt; E[Set saved = await _repository.SaveAsync]
+  E --&gt; F[Return Result.Ok saved]</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>throw new ArgumentNullException(nameof(request));
+var saved = await _repository.SaveAsync(request, ct);</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="n"/>
+    </row>
+    <row r="12" ht="174" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>TC_H_08</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Vong lap long nhau while + do-while, co break thoat vong ngoai</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>public void retrySync(Job job) {
+    int attempt = 0;
+    while (attempt &lt; 3) {
+        do {
+            queue.push(job);
+            attempt++;
+        } while (queue.isFull());
+        if (job.isDone()) {
+            break;
+        }
+    }
+}</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>SLOC=11, V(G)=4 -&gt; ROUTE_HYBRID</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>graph TD
+  A[Start] --&gt; B[Set attempt = 0]
+  B --&gt; C{Loop while attempt &lt; 3?}
+  C -- Yes --&gt; D[Do]
+  D --&gt; E[Push job queue]
+  E --&gt; F[Increase attempt]
+  F --&gt; G{Repeat while queue.isFull?}
+  G -- Yes --&gt; D
+  G -- No --&gt; H{job.isDone?}
+  H -- No --&gt; C
+  C -- No --&gt; I[End]</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>while (attempt &lt; 3) {
+if (job.isDone()) {</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="201" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>TC_H_09</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Class co nhieu ham - moi ham mot do thi con (subgraph) rieng</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>public class OrderValidator {
+    public boolean isValid(Order order) {
+        if (order == null) {
+            return false;
+        }
+        return order.getTotal() &gt; 0;
+    }
+    public void assertValid(Order order) {
+        if (!isValid(order)) {
+            throw new ValidationException("invalid order");
+        }
+    }
+}</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>SLOC=12, V(G)=4 -&gt; ROUTE_HYBRID</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>graph TD
+  subgraph isValid
+  A[Start] --&gt; B{order == null?}
+  B -- Yes --&gt; C[Return false]
+  B -- No --&gt; D[Return order.getTotal &gt; 0]
+  end
+  subgraph assertValid
+  E[Start] --&gt; F{!isValid?}
+  F -- Yes --&gt; G[Throw Validation]
+  end</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>if (order == null) {
+if (!isValid(order)) {
+throw new ValidationException("invalid order");</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="n"/>
+    </row>
+    <row r="14" ht="66" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>TC_H_10</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Ma nguon loi cu phap (thieu dau ngoac) - Tang 2 phai tra HTTP 200, khong duoc treo hay 500</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>public void broken(Order order) {
+    if (order == null {
+        save(order);
+}</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>SLOC=4, V(G)=2 -&gt; ROUTE_HYBRID (AST hasError)</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="106.5" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>TC_H_11</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Comment va chuoi chua ky tu gay nhieu ( ; { } if ) - khong duoc tinh thanh nhanh re</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>public void log(User u) {
+    // if (u == null) throw new Fake();
+    String msg = "user; {id} =&gt; " + u.getId();
+    if (u.isActive()) {
+        auditLogger.info(msg);
+    }
+}</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>SLOC=6, V(G)=2 -&gt; ROUTE_HYBRID</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>graph TD
+  A[Start] --&gt; B[Set msg]
+  B --&gt; C{u.isActive?}
+  C -- Yes --&gt; D[Info auditLogger]
+  C -- No --&gt; E[End]</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>if (u.isActive()) {</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="n"/>
+    </row>
+    <row r="16" ht="66" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>TC_H_12</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Ham tuyen tinh khong nhanh re (dang le di ROUTE_RAW_CODE) - Tang 2 van sinh CFG hop le</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>public String greet(User u) {
+    String name = u.getName();
+    return "Hello " + name;
+}</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>SLOC=4, V(G)=1 -&gt; ROUTE_RAW_CODE</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>graph TD
+  A[Start] --&gt; B[Set name = u.getName]
+  B --&gt; C[Return Hello name]
+  C --&gt; D[End]</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="4" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>

</xml_diff>